<commit_message>
Coordenadas corregidas en Valle y Risaralda; Palmira con 20 sedes en todo el visor
Todo Valle pasa de 97,3 h a 101,0 h. El aumento es por ir a donde estan las
escuelas: El Placer estaba 22,5 km fuera de sitio (en la ciudad de Buga y no en
la cordillera) y Luis Carlos Pena 7 km (en el casco urbano de Cartago y no en
el corregimiento Cauca). Tambien se movieron Panorama e Irene Ferrerosa en
Yumbo, que tenian el mismo punto, Tulio Enrique Tascon, Atanasio Girardot, el
Instituto Tecnico Agricola (a su entrada), Angel Cuadros, Antonio Guendica y
Santa Teresita de Cartago.

Risaralda baja de 45,8 h a 45,6 h con Alto Cauca en su caserio, a 1,1 km del
punto del SIMAT. Su optimo, como el del Valle, vale para el reparto de
municipios que se fijo a mano, y la pantalla lo dice.

El globo de cada municipio y la vista del requerimiento del MEN seguian con
las 21 sedes viejas de Palmira. Ahora usan la lista del 21-sep (20 sedes), y
'en el plan' se cuenta contra los dos planes vigentes: 152 de 485.
</commit_message>
<xml_diff>
--- a/public/datos/plan_cuadrillas_risaralda.xlsx
+++ b/public/datos/plan_cuadrillas_risaralda.xlsx
@@ -2580,7 +2580,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>BASICO OTUN</t>
+          <t>LUIS CARLOS GONZALES MEJIA</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>166170000329</t>
+          <t>166170001490</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>BARRIO SAN JUDAS EL BALSO</t>
+          <t>BARRIO VILLA ALEXANDRA</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2619,13 +2619,13 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>5.75</v>
+        <v>9.4</v>
       </c>
       <c r="Q18" t="n">
-        <v>4.6</v>
+        <v>0.14</v>
       </c>
       <c r="R18" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S18" t="n">
         <v>6.8</v>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>via principal pavimentada</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
@@ -2652,12 +2652,12 @@
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 7 m de esa vía.</t>
+          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 5 m de esa vía.</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>Carrera 19</t>
+          <t>Calle 9</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
@@ -2666,10 +2666,10 @@
         </is>
       </c>
       <c r="AC18" t="n">
-        <v>4.816666667</v>
+        <v>4.823055556</v>
       </c>
       <c r="AD18" t="n">
-        <v>-75.68333333</v>
+        <v>-75.6925</v>
       </c>
     </row>
     <row r="19">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>LUIS CARLOS GONZALES MEJIA</t>
+          <t>INSTITUTO EDUCATIVO EMPRESARIAL</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>166170001490</t>
+          <t>166170001911</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>BARRIO VILLA ALEXANDRA</t>
+          <t>LA BADEA -ANTIGUA  PLAZA DE FERIAS</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2743,20 +2743,20 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>4.6</v>
+        <v>0.14</v>
       </c>
       <c r="Q19" t="n">
-        <v>7.6</v>
+        <v>7.44</v>
       </c>
       <c r="R19" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S19" t="n">
         <v>6.8</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Afectación menor</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
@@ -2776,7 +2776,7 @@
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 5 m de esa vía.</t>
+          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 21 m de esa vía.</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">
@@ -2793,7 +2793,7 @@
         <v>4.823055556</v>
       </c>
       <c r="AD19" t="n">
-        <v>-75.6925</v>
+        <v>-75.69194444</v>
       </c>
     </row>
     <row r="20">
@@ -3343,16 +3343,16 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>34.87</v>
+        <v>28.62</v>
       </c>
       <c r="Q24" t="n">
-        <v>7.8</v>
+        <v>0.96</v>
       </c>
       <c r="R24" t="n">
-        <v>76.90000000000001</v>
+        <v>63.8</v>
       </c>
       <c r="S24" t="n">
-        <v>22.9</v>
+        <v>18.8</v>
       </c>
       <c r="V24" t="inlineStr">
         <is>
@@ -3366,7 +3366,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>camino destapado</t>
+          <t>camino rural sin categoria</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
@@ -3376,19 +3376,24 @@
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 110 m de esa vía.</t>
+          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 2 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>Buena Vista</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AC24" t="n">
-        <v>4.991425841</v>
+        <v>4.994828</v>
       </c>
       <c r="AD24" t="n">
-        <v>-75.75301358</v>
+        <v>-75.743863</v>
       </c>
     </row>
     <row r="25">
@@ -3462,16 +3467,16 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>7.8</v>
+        <v>0.96</v>
       </c>
       <c r="Q25" t="n">
         <v>34.19</v>
       </c>
       <c r="R25" t="n">
-        <v>76.90000000000001</v>
+        <v>63.8</v>
       </c>
       <c r="S25" t="n">
-        <v>22.9</v>
+        <v>18.8</v>
       </c>
       <c r="V25" t="inlineStr">
         <is>
@@ -5263,7 +5268,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>FABIO VASQUEZ BOTERO</t>
+          <t>SAN RAFAEL</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -5273,7 +5278,7 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>166170001023</t>
+          <t>166170001937</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -5288,7 +5293,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>LA PRADERA</t>
+          <t>KR 31 CL 13 SAN RAFAEL</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -5302,25 +5307,25 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>7.14</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="Q40" t="n">
-        <v>3.88</v>
+        <v>3.41</v>
       </c>
       <c r="R40" t="n">
-        <v>18.5</v>
+        <v>22.3</v>
       </c>
       <c r="S40" t="n">
-        <v>7.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Sin afectación</t>
         </is>
       </c>
       <c r="X40" t="inlineStr">
@@ -5335,7 +5340,7 @@
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 16 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 2 m de esa vía.</t>
         </is>
       </c>
       <c r="AB40" t="inlineStr">
@@ -5344,10 +5349,10 @@
         </is>
       </c>
       <c r="AC40" t="n">
-        <v>4.830277778</v>
+        <v>4.817222222</v>
       </c>
       <c r="AD40" t="n">
-        <v>-75.6825</v>
+        <v>-75.6725</v>
       </c>
     </row>
     <row r="41">
@@ -5382,17 +5387,17 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>INSTITUTO EDUCATIVO EMPRESARIAL</t>
+          <t>LUIS CARLOS GALAN SARMIENTO</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA EMPRESARIAL</t>
+          <t>INSTITUCION EDUCATIVA POPULAR DIOCESANO</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>166170001911</t>
+          <t>166170001481</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -5407,7 +5412,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>LA BADEA -ANTIGUA  PLAZA DE FERIAS</t>
+          <t>BARRIO LAS VEGAS</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -5421,20 +5426,20 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>3.88</v>
+        <v>3.41</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.44</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="R41" t="n">
-        <v>18.5</v>
+        <v>22.3</v>
       </c>
       <c r="S41" t="n">
-        <v>7.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>Afectación menor</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W41" t="inlineStr">
@@ -5444,7 +5449,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>via principal pavimentada</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -5454,12 +5459,12 @@
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 21 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 13 m de esa vía.</t>
         </is>
       </c>
       <c r="AA41" t="inlineStr">
         <is>
-          <t>Calle 9</t>
+          <t>Carrera 24A</t>
         </is>
       </c>
       <c r="AB41" t="inlineStr">
@@ -5468,10 +5473,10 @@
         </is>
       </c>
       <c r="AC41" t="n">
-        <v>4.823055556</v>
+        <v>4.816944444</v>
       </c>
       <c r="AD41" t="n">
-        <v>-75.69194444</v>
+        <v>-75.67805556</v>
       </c>
     </row>
     <row r="42">
@@ -5744,7 +5749,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>SAN RAFAEL</t>
+          <t>FABIO VASQUEZ BOTERO</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -5754,7 +5759,7 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>166170001937</t>
+          <t>166170001023</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -5769,7 +5774,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>KR 31 CL 13 SAN RAFAEL</t>
+          <t>LA PRADERA</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -5783,25 +5788,25 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>9.470000000000001</v>
+        <v>7.14</v>
       </c>
       <c r="Q44" t="n">
-        <v>3.41</v>
+        <v>5.72</v>
       </c>
       <c r="R44" t="n">
-        <v>22.3</v>
+        <v>19.5</v>
       </c>
       <c r="S44" t="n">
-        <v>8.199999999999999</v>
+        <v>7.4</v>
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>Sin afectación</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X44" t="inlineStr">
@@ -5816,7 +5821,7 @@
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 2 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 16 m de esa vía.</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5825,10 +5830,10 @@
         </is>
       </c>
       <c r="AC44" t="n">
-        <v>4.817222222</v>
+        <v>4.830277778</v>
       </c>
       <c r="AD44" t="n">
-        <v>-75.6725</v>
+        <v>-75.6825</v>
       </c>
     </row>
     <row r="45">
@@ -5863,17 +5868,17 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>LUIS CARLOS GALAN SARMIENTO</t>
+          <t>BASICO OTUN</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA POPULAR DIOCESANO</t>
+          <t>INSTITUCION EDUCATIVA EMPRESARIAL</t>
         </is>
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>166170001481</t>
+          <t>166170000329</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -5888,7 +5893,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>BARRIO LAS VEGAS</t>
+          <t>BARRIO SAN JUDAS EL BALSO</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -5902,16 +5907,16 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>3.41</v>
+        <v>5.72</v>
       </c>
       <c r="Q45" t="n">
-        <v>9.460000000000001</v>
+        <v>6.63</v>
       </c>
       <c r="R45" t="n">
-        <v>22.3</v>
+        <v>19.5</v>
       </c>
       <c r="S45" t="n">
-        <v>8.199999999999999</v>
+        <v>7.4</v>
       </c>
       <c r="V45" t="inlineStr">
         <is>
@@ -5935,12 +5940,12 @@
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 13 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 7 m de esa vía.</t>
         </is>
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>Carrera 24A</t>
+          <t>Carrera 19</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5949,10 +5954,10 @@
         </is>
       </c>
       <c r="AC45" t="n">
-        <v>4.816944444</v>
+        <v>4.816666667</v>
       </c>
       <c r="AD45" t="n">
-        <v>-75.67805556</v>
+        <v>-75.68333333</v>
       </c>
     </row>
     <row r="46">
@@ -8161,7 +8166,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -8300,10 +8305,10 @@
         <v>28</v>
       </c>
       <c r="D11" t="n">
-        <v>9.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="F11" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Sin textos de rectores, estado alineado en los Excel y areas del predio bajo el punto
- Fuera las observaciones y acciones de los rectores, que la Secretaria del
  Valle retiro de su tablero el 21-sep (Ley 1581). Las fotos siguen.
- Excel del plan: «No reportó al MEN» en vez de «Sin afectación», y columnas
  de FFIE, reporte a la Secretaria, restriccion de la ficha, marca del mapa y
  especialidad de la visita.
- Area de terreno y construida del predio que queda bajo el punto actual, solo
  cuando hay respaldo de que es la escuela.
</commit_message>
<xml_diff>
--- a/public/datos/plan_cuadrillas_risaralda.xlsx
+++ b/public/datos/plan_cuadrillas_risaralda.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan'!$A$1:$AD$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Plan'!$A$1:$AI$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD63"/>
+  <dimension ref="A1:AI63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,55 +550,80 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Concepto (tablero del Valle)</t>
+          <t>Especialidad de la visita</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
+          <t>Concepto técnico (tablero del Valle)</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
           <t>Dictamen</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Estado (MEN)</t>
-        </is>
-      </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
+          <t>Restringido en la ficha</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Reporte rector al MEN</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
           <t>Nivel de afectación (MEN)</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Reporte rector a la Secretaría del Valle</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Reporte FFIE 2026</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Marca en el mapa</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Tipo de vía</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Acceso</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Por qué</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Vía de acceso</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Coordenada en revisión</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Latitud</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Longitud</t>
         </is>
@@ -686,45 +711,45 @@
       <c r="S2" t="n">
         <v>64.3</v>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X2" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 6 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Carrera 7</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC2" t="n">
+      <c r="AH2" t="n">
         <v>5.104722222</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AI2" t="n">
         <v>-75.9425</v>
       </c>
     </row>
@@ -810,40 +835,40 @@
       <c r="S3" t="n">
         <v>90.5</v>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>Colapso parcial</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>camino destapado</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AE3" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 240 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="AC3" t="n">
+      <c r="AH3" t="n">
         <v>5.331280525</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AI3" t="n">
         <v>-75.9852455</v>
       </c>
     </row>
@@ -929,45 +954,45 @@
       <c r="S4" t="n">
         <v>0.8</v>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>Colapso parcial</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 8 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>Calle 3 A</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="AC4" t="n">
+      <c r="AH4" t="n">
         <v>5.21916175028</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AI4" t="n">
         <v>-76.0331189595</v>
       </c>
     </row>
@@ -1053,45 +1078,45 @@
       <c r="S5" t="n">
         <v>67</v>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X5" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>rojo</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AE5" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 20 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>Calle 3</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
+      <c r="AG5" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC5" t="n">
+      <c r="AH5" t="n">
         <v>5.340317929</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AI5" t="n">
         <v>-76.14533188999999</v>
       </c>
     </row>
@@ -1177,40 +1202,40 @@
       <c r="S6" t="n">
         <v>67</v>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AE6" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 58 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AG6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC6" t="n">
+      <c r="AH6" t="n">
         <v>5.366205</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AI6" t="n">
         <v>-76.10596200000001</v>
       </c>
     </row>
@@ -1296,40 +1321,40 @@
       <c r="S7" t="n">
         <v>74.09999999999999</v>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>via principal pavimentada</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="AE7" t="inlineStr">
         <is>
           <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «primary»). La sede queda a 3687 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
+      <c r="AG7" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="AC7" t="n">
+      <c r="AH7" t="n">
         <v>5.312197</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AI7" t="n">
         <v>-76.166676</v>
       </c>
     </row>
@@ -1415,40 +1440,40 @@
       <c r="S8" t="n">
         <v>74.09999999999999</v>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>via principal pavimentada</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr">
+      <c r="AE8" t="inlineStr">
         <is>
           <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «primary»). La sede queda a 281 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
+      <c r="AG8" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC8" t="n">
+      <c r="AH8" t="n">
         <v>5.355261</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AI8" t="n">
         <v>-76.177787</v>
       </c>
     </row>
@@ -1534,40 +1559,40 @@
       <c r="S9" t="n">
         <v>79.3</v>
       </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X9" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
           <t>otra</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="AD9" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
+      <c r="AE9" t="inlineStr">
         <is>
           <t>La vía de entrada es otra según OpenStreetMap (clase «track_grade3»). La sede queda a 5445 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB9" t="inlineStr">
+      <c r="AG9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC9" t="n">
+      <c r="AH9" t="n">
         <v>5.275278</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AI9" t="n">
         <v>-76.162778</v>
       </c>
     </row>
@@ -1653,45 +1678,45 @@
       <c r="S10" t="n">
         <v>35.5</v>
       </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X10" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
           <t>via terciaria</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="AD10" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr">
+      <c r="AE10" t="inlineStr">
         <is>
           <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 75 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr">
+      <c r="AF10" t="inlineStr">
         <is>
           <t>Mateguadua-Apia</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
+      <c r="AG10" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="AC10" t="n">
+      <c r="AH10" t="n">
         <v>5.11777777778</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AI10" t="n">
         <v>-75.90472222219999</v>
       </c>
     </row>
@@ -1777,40 +1802,40 @@
       <c r="S11" t="n">
         <v>35.5</v>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>Colapso parcial</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>otra</t>
         </is>
       </c>
-      <c r="Y11" t="inlineStr">
+      <c r="AD11" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr">
+      <c r="AE11" t="inlineStr">
         <is>
           <t>La vía de entrada es otra según OpenStreetMap (clase «track_grade3»). La sede queda a 293 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB11" t="inlineStr">
+      <c r="AG11" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC11" t="n">
+      <c r="AH11" t="n">
         <v>5.151535</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AI11" t="n">
         <v>-75.904819</v>
       </c>
     </row>
@@ -1896,40 +1921,45 @@
       <c r="S12" t="n">
         <v>10.5</v>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="X12" t="inlineStr">
         <is>
           <t>Colapso total</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="Y12" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>rojo</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
+      <c r="AD12" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
+      <c r="AE12" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 44 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
+      <c r="AG12" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC12" t="n">
+      <c r="AH12" t="n">
         <v>5.165871128</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AI12" t="n">
         <v>-75.86350014999999</v>
       </c>
     </row>
@@ -2015,40 +2045,40 @@
       <c r="S13" t="n">
         <v>10.5</v>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="AC13" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
+      <c r="AD13" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z13" t="inlineStr">
+      <c r="AE13" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 2 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr">
+      <c r="AG13" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC13" t="n">
+      <c r="AH13" t="n">
         <v>5.165833</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AI13" t="n">
         <v>-75.864133</v>
       </c>
     </row>
@@ -2134,40 +2164,40 @@
       <c r="S14" t="n">
         <v>42.4</v>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
+      <c r="AC14" t="inlineStr">
         <is>
           <t>camino destapado</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
+      <c r="AD14" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr">
+      <c r="AE14" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 8 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB14" t="inlineStr">
+      <c r="AG14" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC14" t="n">
+      <c r="AH14" t="n">
         <v>5.174781</v>
       </c>
-      <c r="AD14" t="n">
+      <c r="AI14" t="n">
         <v>-75.89761</v>
       </c>
     </row>
@@ -2253,40 +2283,40 @@
       <c r="S15" t="n">
         <v>42.4</v>
       </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X15" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
           <t>via terciaria</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="AD15" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z15" t="inlineStr">
+      <c r="AE15" t="inlineStr">
         <is>
           <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 11 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB15" t="inlineStr">
+      <c r="AG15" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC15" t="n">
+      <c r="AH15" t="n">
         <v>5.279785869</v>
       </c>
-      <c r="AD15" t="n">
+      <c r="AI15" t="n">
         <v>-75.89025909</v>
       </c>
     </row>
@@ -2372,45 +2402,45 @@
       <c r="S16" t="n">
         <v>43.4</v>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr">
+      <c r="Y16" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="AC16" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="AD16" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z16" t="inlineStr">
+      <c r="AE16" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 4 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA16" t="inlineStr">
+      <c r="AF16" t="inlineStr">
         <is>
           <t>Carrera 4</t>
         </is>
       </c>
-      <c r="AB16" t="inlineStr">
+      <c r="AG16" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC16" t="n">
+      <c r="AH16" t="n">
         <v>5.30751835</v>
       </c>
-      <c r="AD16" t="n">
+      <c r="AI16" t="n">
         <v>-75.82041798</v>
       </c>
     </row>
@@ -2496,45 +2526,50 @@
       <c r="S17" t="n">
         <v>43.4</v>
       </c>
-      <c r="V17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr">
+      <c r="Y17" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>rojo</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
         <is>
           <t>via terciaria</t>
         </is>
       </c>
-      <c r="Y17" t="inlineStr">
+      <c r="AD17" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z17" t="inlineStr">
+      <c r="AE17" t="inlineStr">
         <is>
           <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 13 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA17" t="inlineStr">
+      <c r="AF17" t="inlineStr">
         <is>
           <t>Calle 12</t>
         </is>
       </c>
-      <c r="AB17" t="inlineStr">
+      <c r="AG17" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC17" t="n">
+      <c r="AH17" t="n">
         <v>5.318849336</v>
       </c>
-      <c r="AD17" t="n">
+      <c r="AI17" t="n">
         <v>-75.80047681000001</v>
       </c>
     </row>
@@ -2620,40 +2655,40 @@
       <c r="S18" t="n">
         <v>19.2</v>
       </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X18" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y18" t="inlineStr">
+      <c r="AD18" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z18" t="inlineStr">
+      <c r="AE18" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 199 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB18" t="inlineStr">
+      <c r="AG18" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC18" t="n">
+      <c r="AH18" t="n">
         <v>5.328055556</v>
       </c>
-      <c r="AD18" t="n">
+      <c r="AI18" t="n">
         <v>-75.74833332999999</v>
       </c>
     </row>
@@ -2739,40 +2774,40 @@
       <c r="S19" t="n">
         <v>19.2</v>
       </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X19" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr">
+      <c r="AD19" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z19" t="inlineStr">
+      <c r="AE19" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 36 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB19" t="inlineStr">
+      <c r="AG19" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC19" t="n">
+      <c r="AH19" t="n">
         <v>5.370566</v>
       </c>
-      <c r="AD19" t="n">
+      <c r="AI19" t="n">
         <v>-75.74896699999999</v>
       </c>
     </row>
@@ -2858,40 +2893,40 @@
       <c r="S20" t="n">
         <v>32.6</v>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W20" t="inlineStr">
+      <c r="Y20" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr">
+      <c r="AC20" t="inlineStr">
         <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y20" t="inlineStr">
+      <c r="AD20" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z20" t="inlineStr">
+      <c r="AE20" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 8 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB20" t="inlineStr">
+      <c r="AG20" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC20" t="n">
+      <c r="AH20" t="n">
         <v>5.283929</v>
       </c>
-      <c r="AD20" t="n">
+      <c r="AI20" t="n">
         <v>-75.69113299999999</v>
       </c>
     </row>
@@ -2977,45 +3012,45 @@
       <c r="S21" t="n">
         <v>89.7</v>
       </c>
-      <c r="V21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>Colapso parcial</t>
         </is>
       </c>
-      <c r="W21" t="inlineStr">
+      <c r="Y21" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr">
+      <c r="AC21" t="inlineStr">
         <is>
           <t>via terciaria</t>
         </is>
       </c>
-      <c r="Y21" t="inlineStr">
+      <c r="AD21" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z21" t="inlineStr">
+      <c r="AE21" t="inlineStr">
         <is>
           <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 19 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA21" t="inlineStr">
+      <c r="AF21" t="inlineStr">
         <is>
           <t>Via Irra a Quinchia</t>
         </is>
       </c>
-      <c r="AB21" t="inlineStr">
+      <c r="AG21" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC21" t="n">
+      <c r="AH21" t="n">
         <v>5.29672</v>
       </c>
-      <c r="AD21" t="n">
+      <c r="AI21" t="n">
         <v>-75.66537599999999</v>
       </c>
     </row>
@@ -3101,45 +3136,45 @@
       <c r="S22" t="n">
         <v>6.8</v>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W22" t="inlineStr">
+      <c r="Y22" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr">
+      <c r="AC22" t="inlineStr">
         <is>
           <t>via principal pavimentada</t>
         </is>
       </c>
-      <c r="Y22" t="inlineStr">
+      <c r="AD22" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z22" t="inlineStr">
+      <c r="AE22" t="inlineStr">
         <is>
           <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 5 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA22" t="inlineStr">
+      <c r="AF22" t="inlineStr">
         <is>
           <t>Calle 9</t>
         </is>
       </c>
-      <c r="AB22" t="inlineStr">
+      <c r="AG22" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC22" t="n">
+      <c r="AH22" t="n">
         <v>4.823055556</v>
       </c>
-      <c r="AD22" t="n">
+      <c r="AI22" t="n">
         <v>-75.6925</v>
       </c>
     </row>
@@ -3225,45 +3260,45 @@
       <c r="S23" t="n">
         <v>6.8</v>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W23" t="inlineStr">
+      <c r="Y23" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr">
+      <c r="AC23" t="inlineStr">
         <is>
           <t>via principal pavimentada</t>
         </is>
       </c>
-      <c r="Y23" t="inlineStr">
+      <c r="AD23" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z23" t="inlineStr">
+      <c r="AE23" t="inlineStr">
         <is>
           <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 21 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA23" t="inlineStr">
+      <c r="AF23" t="inlineStr">
         <is>
           <t>Calle 9</t>
         </is>
       </c>
-      <c r="AB23" t="inlineStr">
+      <c r="AG23" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC23" t="n">
+      <c r="AH23" t="n">
         <v>4.823055556</v>
       </c>
-      <c r="AD23" t="n">
+      <c r="AI23" t="n">
         <v>-75.69194444</v>
       </c>
     </row>
@@ -3349,40 +3384,45 @@
       <c r="S24" t="n">
         <v>9</v>
       </c>
-      <c r="V24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>Colapso parcial</t>
         </is>
       </c>
-      <c r="W24" t="inlineStr">
+      <c r="Y24" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr">
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>rojo</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y24" t="inlineStr">
+      <c r="AD24" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z24" t="inlineStr">
+      <c r="AE24" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 6 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB24" t="inlineStr">
+      <c r="AG24" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC24" t="n">
+      <c r="AH24" t="n">
         <v>4.824166667</v>
       </c>
-      <c r="AD24" t="n">
+      <c r="AI24" t="n">
         <v>-75.69972222</v>
       </c>
     </row>
@@ -3468,40 +3508,40 @@
       <c r="S25" t="n">
         <v>9</v>
       </c>
-      <c r="V25" t="inlineStr">
+      <c r="X25" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W25" t="inlineStr">
+      <c r="Y25" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr">
+      <c r="AC25" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y25" t="inlineStr">
+      <c r="AD25" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z25" t="inlineStr">
+      <c r="AE25" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 20 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB25" t="inlineStr">
+      <c r="AG25" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="AC25" t="n">
+      <c r="AH25" t="n">
         <v>4.82381384716</v>
       </c>
-      <c r="AD25" t="n">
+      <c r="AI25" t="n">
         <v>-75.699591841</v>
       </c>
     </row>
@@ -3587,40 +3627,40 @@
       <c r="S26" t="n">
         <v>35.5</v>
       </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X26" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y26" t="inlineStr">
+      <c r="AD26" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z26" t="inlineStr">
+      <c r="AE26" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 35 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB26" t="inlineStr">
+      <c r="AG26" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC26" t="n">
+      <c r="AH26" t="n">
         <v>4.9022</v>
       </c>
-      <c r="AD26" t="n">
+      <c r="AI26" t="n">
         <v>-75.773707</v>
       </c>
     </row>
@@ -3706,40 +3746,40 @@
       <c r="S27" t="n">
         <v>35.5</v>
       </c>
-      <c r="V27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W27" t="inlineStr">
+      <c r="Y27" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr">
+      <c r="AC27" t="inlineStr">
         <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y27" t="inlineStr">
+      <c r="AD27" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z27" t="inlineStr">
+      <c r="AE27" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 40 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB27" t="inlineStr">
+      <c r="AG27" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC27" t="n">
+      <c r="AH27" t="n">
         <v>4.928985175</v>
       </c>
-      <c r="AD27" t="n">
+      <c r="AI27" t="n">
         <v>-75.77832192</v>
       </c>
     </row>
@@ -3825,45 +3865,50 @@
       <c r="S28" t="n">
         <v>18.8</v>
       </c>
-      <c r="V28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>Riesgo inminente de colapso</t>
         </is>
       </c>
-      <c r="W28" t="inlineStr">
+      <c r="Y28" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr">
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>rojo</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
         <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y28" t="inlineStr">
+      <c r="AD28" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z28" t="inlineStr">
+      <c r="AE28" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 2 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA28" t="inlineStr">
+      <c r="AF28" t="inlineStr">
         <is>
           <t>Buena Vista</t>
         </is>
       </c>
-      <c r="AB28" t="inlineStr">
+      <c r="AG28" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC28" t="n">
+      <c r="AH28" t="n">
         <v>4.994828</v>
       </c>
-      <c r="AD28" t="n">
+      <c r="AI28" t="n">
         <v>-75.743863</v>
       </c>
     </row>
@@ -3949,45 +3994,45 @@
       <c r="S29" t="n">
         <v>18.8</v>
       </c>
-      <c r="V29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W29" t="inlineStr">
+      <c r="Y29" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr">
+      <c r="AC29" t="inlineStr">
         <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y29" t="inlineStr">
+      <c r="AD29" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z29" t="inlineStr">
+      <c r="AE29" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 7 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA29" t="inlineStr">
+      <c r="AF29" t="inlineStr">
         <is>
           <t>Buena Vista</t>
         </is>
       </c>
-      <c r="AB29" t="inlineStr">
+      <c r="AG29" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC29" t="n">
+      <c r="AH29" t="n">
         <v>4.992762</v>
       </c>
-      <c r="AD29" t="n">
+      <c r="AI29" t="n">
         <v>-75.74432</v>
       </c>
     </row>
@@ -4073,40 +4118,40 @@
       <c r="S30" t="n">
         <v>26.6</v>
       </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W30" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X30" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y30" t="inlineStr">
+      <c r="AD30" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z30" t="inlineStr">
+      <c r="AE30" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 22 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB30" t="inlineStr">
+      <c r="AG30" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="AC30" t="n">
+      <c r="AH30" t="n">
         <v>4.909338798</v>
       </c>
-      <c r="AD30" t="n">
+      <c r="AI30" t="n">
         <v>-75.72299636</v>
       </c>
     </row>
@@ -4192,45 +4237,45 @@
       <c r="S31" t="n">
         <v>26.6</v>
       </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X31" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y31" t="inlineStr">
+      <c r="AD31" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z31" t="inlineStr">
+      <c r="AE31" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 318 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA31" t="inlineStr">
+      <c r="AF31" t="inlineStr">
         <is>
           <t>Vía la Bodega</t>
         </is>
       </c>
-      <c r="AB31" t="inlineStr">
+      <c r="AG31" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="AC31" t="n">
+      <c r="AH31" t="n">
         <v>4.896608682</v>
       </c>
-      <c r="AD31" t="n">
+      <c r="AI31" t="n">
         <v>-75.71433512</v>
       </c>
     </row>
@@ -4316,45 +4361,45 @@
       <c r="S32" t="n">
         <v>1.4</v>
       </c>
-      <c r="V32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W32" t="inlineStr">
+      <c r="Y32" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr">
+      <c r="AC32" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y32" t="inlineStr">
+      <c r="AD32" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z32" t="inlineStr">
+      <c r="AE32" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 18 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA32" t="inlineStr">
+      <c r="AF32" t="inlineStr">
         <is>
           <t>Carrera 18</t>
         </is>
       </c>
-      <c r="AB32" t="inlineStr">
+      <c r="AG32" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC32" t="n">
+      <c r="AH32" t="n">
         <v>4.835834367</v>
       </c>
-      <c r="AD32" t="n">
+      <c r="AI32" t="n">
         <v>-75.66730004</v>
       </c>
     </row>
@@ -4440,45 +4485,45 @@
       <c r="S33" t="n">
         <v>2.4</v>
       </c>
-      <c r="V33" t="inlineStr">
+      <c r="X33" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W33" t="inlineStr">
+      <c r="Y33" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="X33" t="inlineStr">
+      <c r="AC33" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y33" t="inlineStr">
+      <c r="AD33" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z33" t="inlineStr">
+      <c r="AE33" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 23 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA33" t="inlineStr">
+      <c r="AF33" t="inlineStr">
         <is>
           <t>Calle 61</t>
         </is>
       </c>
-      <c r="AB33" t="inlineStr">
+      <c r="AG33" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC33" t="n">
+      <c r="AH33" t="n">
         <v>4.843896232</v>
       </c>
-      <c r="AD33" t="n">
+      <c r="AI33" t="n">
         <v>-75.66503904</v>
       </c>
     </row>
@@ -4564,45 +4609,45 @@
       <c r="S34" t="n">
         <v>2.1</v>
       </c>
-      <c r="V34" t="inlineStr">
+      <c r="X34" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W34" t="inlineStr">
+      <c r="Y34" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="X34" t="inlineStr">
+      <c r="AC34" t="inlineStr">
         <is>
           <t>via terciaria</t>
         </is>
       </c>
-      <c r="Y34" t="inlineStr">
+      <c r="AD34" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z34" t="inlineStr">
+      <c r="AE34" t="inlineStr">
         <is>
           <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 12 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA34" t="inlineStr">
+      <c r="AF34" t="inlineStr">
         <is>
           <t>Carrera 21</t>
         </is>
       </c>
-      <c r="AB34" t="inlineStr">
+      <c r="AG34" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC34" t="n">
+      <c r="AH34" t="n">
         <v>4.833675657</v>
       </c>
-      <c r="AD34" t="n">
+      <c r="AI34" t="n">
         <v>-75.66815895000001</v>
       </c>
     </row>
@@ -4688,45 +4733,45 @@
       <c r="S35" t="n">
         <v>2.1</v>
       </c>
-      <c r="V35" t="inlineStr">
+      <c r="X35" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W35" t="inlineStr">
+      <c r="Y35" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="X35" t="inlineStr">
+      <c r="AC35" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y35" t="inlineStr">
+      <c r="AD35" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z35" t="inlineStr">
+      <c r="AE35" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 4 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA35" t="inlineStr">
+      <c r="AF35" t="inlineStr">
         <is>
           <t>Carrera 23</t>
         </is>
       </c>
-      <c r="AB35" t="inlineStr">
+      <c r="AG35" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC35" t="n">
+      <c r="AH35" t="n">
         <v>4.834166667</v>
       </c>
-      <c r="AD35" t="n">
+      <c r="AI35" t="n">
         <v>-75.66527778</v>
       </c>
     </row>
@@ -4812,45 +4857,45 @@
       <c r="S36" t="n">
         <v>3</v>
       </c>
-      <c r="V36" t="inlineStr">
+      <c r="X36" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W36" t="inlineStr">
+      <c r="Y36" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr">
+      <c r="AC36" t="inlineStr">
         <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y36" t="inlineStr">
+      <c r="AD36" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z36" t="inlineStr">
+      <c r="AE36" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 17 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA36" t="inlineStr">
+      <c r="AF36" t="inlineStr">
         <is>
           <t>Calle 64</t>
         </is>
       </c>
-      <c r="AB36" t="inlineStr">
+      <c r="AG36" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC36" t="n">
+      <c r="AH36" t="n">
         <v>4.843075404</v>
       </c>
-      <c r="AD36" t="n">
+      <c r="AI36" t="n">
         <v>-75.66069447</v>
       </c>
     </row>
@@ -4936,45 +4981,45 @@
       <c r="S37" t="n">
         <v>3</v>
       </c>
-      <c r="V37" t="inlineStr">
+      <c r="X37" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W37" t="inlineStr">
+      <c r="Y37" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="X37" t="inlineStr">
+      <c r="AC37" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y37" t="inlineStr">
+      <c r="AD37" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z37" t="inlineStr">
+      <c r="AE37" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 11 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA37" t="inlineStr">
+      <c r="AF37" t="inlineStr">
         <is>
           <t>Calle 67</t>
         </is>
       </c>
-      <c r="AB37" t="inlineStr">
+      <c r="AG37" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC37" t="n">
+      <c r="AH37" t="n">
         <v>4.844819</v>
       </c>
-      <c r="AD37" t="n">
+      <c r="AI37" t="n">
         <v>-75.660687</v>
       </c>
     </row>
@@ -5060,45 +5105,45 @@
       <c r="S38" t="n">
         <v>8</v>
       </c>
-      <c r="V38" t="inlineStr">
+      <c r="X38" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W38" t="inlineStr">
+      <c r="Y38" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X38" t="inlineStr">
+      <c r="AC38" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y38" t="inlineStr">
+      <c r="AD38" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z38" t="inlineStr">
+      <c r="AE38" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 13 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA38" t="inlineStr">
+      <c r="AF38" t="inlineStr">
         <is>
           <t>Carrera 24A</t>
         </is>
       </c>
-      <c r="AB38" t="inlineStr">
+      <c r="AG38" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC38" t="n">
+      <c r="AH38" t="n">
         <v>4.816944444</v>
       </c>
-      <c r="AD38" t="n">
+      <c r="AI38" t="n">
         <v>-75.67805556</v>
       </c>
     </row>
@@ -5184,40 +5229,40 @@
       <c r="S39" t="n">
         <v>8</v>
       </c>
-      <c r="V39" t="inlineStr">
+      <c r="X39" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W39" t="inlineStr">
+      <c r="Y39" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X39" t="inlineStr">
+      <c r="AC39" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y39" t="inlineStr">
+      <c r="AD39" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z39" t="inlineStr">
+      <c r="AE39" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 2 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB39" t="inlineStr">
+      <c r="AG39" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC39" t="n">
+      <c r="AH39" t="n">
         <v>4.817222222</v>
       </c>
-      <c r="AD39" t="n">
+      <c r="AI39" t="n">
         <v>-75.6725</v>
       </c>
     </row>
@@ -5303,40 +5348,40 @@
       <c r="S40" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="V40" t="inlineStr">
+      <c r="X40" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W40" t="inlineStr">
+      <c r="Y40" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr">
+      <c r="AC40" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y40" t="inlineStr">
+      <c r="AD40" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z40" t="inlineStr">
+      <c r="AE40" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 56 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB40" t="inlineStr">
+      <c r="AG40" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC40" t="n">
+      <c r="AH40" t="n">
         <v>4.818297979</v>
       </c>
-      <c r="AD40" t="n">
+      <c r="AI40" t="n">
         <v>-75.66450766</v>
       </c>
     </row>
@@ -5422,40 +5467,40 @@
       <c r="S41" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="V41" t="inlineStr">
+      <c r="X41" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W41" t="inlineStr">
+      <c r="Y41" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr">
+      <c r="AC41" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y41" t="inlineStr">
+      <c r="AD41" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z41" t="inlineStr">
+      <c r="AE41" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 36 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB41" t="inlineStr">
+      <c r="AG41" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC41" t="n">
+      <c r="AH41" t="n">
         <v>4.825547182</v>
       </c>
-      <c r="AD41" t="n">
+      <c r="AI41" t="n">
         <v>-75.66634138000001</v>
       </c>
     </row>
@@ -5541,40 +5586,40 @@
       <c r="S42" t="n">
         <v>7.4</v>
       </c>
-      <c r="V42" t="inlineStr">
+      <c r="X42" t="inlineStr">
         <is>
           <t>Colapso parcial</t>
         </is>
       </c>
-      <c r="W42" t="inlineStr">
+      <c r="Y42" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X42" t="inlineStr">
+      <c r="AC42" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y42" t="inlineStr">
+      <c r="AD42" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z42" t="inlineStr">
+      <c r="AE42" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 16 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB42" t="inlineStr">
+      <c r="AG42" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC42" t="n">
+      <c r="AH42" t="n">
         <v>4.830277778</v>
       </c>
-      <c r="AD42" t="n">
+      <c r="AI42" t="n">
         <v>-75.6825</v>
       </c>
     </row>
@@ -5660,45 +5705,45 @@
       <c r="S43" t="n">
         <v>7.4</v>
       </c>
-      <c r="V43" t="inlineStr">
+      <c r="X43" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W43" t="inlineStr">
+      <c r="Y43" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X43" t="inlineStr">
+      <c r="AC43" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y43" t="inlineStr">
+      <c r="AD43" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z43" t="inlineStr">
+      <c r="AE43" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 7 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA43" t="inlineStr">
+      <c r="AF43" t="inlineStr">
         <is>
           <t>Carrera 19</t>
         </is>
       </c>
-      <c r="AB43" t="inlineStr">
+      <c r="AG43" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC43" t="n">
+      <c r="AH43" t="n">
         <v>4.816666667</v>
       </c>
-      <c r="AD43" t="n">
+      <c r="AI43" t="n">
         <v>-75.68333333</v>
       </c>
     </row>
@@ -5784,45 +5829,45 @@
       <c r="S44" t="n">
         <v>5.7</v>
       </c>
-      <c r="V44" t="inlineStr">
+      <c r="X44" t="inlineStr">
         <is>
           <t>Colapso parcial</t>
         </is>
       </c>
-      <c r="W44" t="inlineStr">
+      <c r="Y44" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X44" t="inlineStr">
+      <c r="AC44" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y44" t="inlineStr">
+      <c r="AD44" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z44" t="inlineStr">
+      <c r="AE44" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 15 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA44" t="inlineStr">
+      <c r="AF44" t="inlineStr">
         <is>
           <t>Carrera 5</t>
         </is>
       </c>
-      <c r="AB44" t="inlineStr">
+      <c r="AG44" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC44" t="n">
+      <c r="AH44" t="n">
         <v>4.818122534</v>
       </c>
-      <c r="AD44" t="n">
+      <c r="AI44" t="n">
         <v>-75.71553498</v>
       </c>
     </row>
@@ -5908,45 +5953,45 @@
       <c r="S45" t="n">
         <v>5.7</v>
       </c>
-      <c r="V45" t="inlineStr">
+      <c r="X45" t="inlineStr">
         <is>
           <t>Colapso parcial</t>
         </is>
       </c>
-      <c r="W45" t="inlineStr">
+      <c r="Y45" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X45" t="inlineStr">
+      <c r="AC45" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y45" t="inlineStr">
+      <c r="AD45" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z45" t="inlineStr">
+      <c r="AE45" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 2 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA45" t="inlineStr">
+      <c r="AF45" t="inlineStr">
         <is>
           <t>Carrera 2 Bis</t>
         </is>
       </c>
-      <c r="AB45" t="inlineStr">
+      <c r="AG45" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC45" t="n">
+      <c r="AH45" t="n">
         <v>4.819868522229693</v>
       </c>
-      <c r="AD45" t="n">
+      <c r="AI45" t="n">
         <v>-75.70621902228969</v>
       </c>
     </row>
@@ -6032,40 +6077,40 @@
       <c r="S46" t="n">
         <v>14.1</v>
       </c>
-      <c r="V46" t="inlineStr">
+      <c r="X46" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W46" t="inlineStr">
+      <c r="Y46" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="X46" t="inlineStr">
+      <c r="AC46" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y46" t="inlineStr">
+      <c r="AD46" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z46" t="inlineStr">
+      <c r="AE46" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 5 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB46" t="inlineStr">
+      <c r="AG46" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC46" t="n">
+      <c r="AH46" t="n">
         <v>4.805705</v>
       </c>
-      <c r="AD46" t="n">
+      <c r="AI46" t="n">
         <v>-75.73962299999999</v>
       </c>
     </row>
@@ -6151,45 +6196,45 @@
       <c r="S47" t="n">
         <v>14.1</v>
       </c>
-      <c r="V47" t="inlineStr">
+      <c r="X47" t="inlineStr">
         <is>
           <t>Afectación menor</t>
         </is>
       </c>
-      <c r="W47" t="inlineStr">
+      <c r="Y47" t="inlineStr">
         <is>
           <t>Bajo</t>
         </is>
       </c>
-      <c r="X47" t="inlineStr">
+      <c r="AC47" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y47" t="inlineStr">
+      <c r="AD47" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z47" t="inlineStr">
+      <c r="AE47" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 35 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA47" t="inlineStr">
+      <c r="AF47" t="inlineStr">
         <is>
           <t>Calle 75</t>
         </is>
       </c>
-      <c r="AB47" t="inlineStr">
+      <c r="AG47" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC47" t="n">
+      <c r="AH47" t="n">
         <v>4.803217136</v>
       </c>
-      <c r="AD47" t="n">
+      <c r="AI47" t="n">
         <v>-75.74425404</v>
       </c>
     </row>
@@ -6275,40 +6320,40 @@
       <c r="S48" t="n">
         <v>78.90000000000001</v>
       </c>
-      <c r="V48" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W48" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X48" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB48" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC48" t="inlineStr">
+        <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y48" t="inlineStr">
+      <c r="AD48" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z48" t="inlineStr">
+      <c r="AE48" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 12 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB48" t="inlineStr">
+      <c r="AG48" t="inlineStr">
         <is>
           <t>sí</t>
         </is>
       </c>
-      <c r="AC48" t="n">
+      <c r="AH48" t="n">
         <v>4.99014911697</v>
       </c>
-      <c r="AD48" t="n">
+      <c r="AI48" t="n">
         <v>-75.9242208477</v>
       </c>
     </row>
@@ -6394,40 +6439,40 @@
       <c r="S49" t="n">
         <v>42.5</v>
       </c>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W49" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X49" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC49" t="inlineStr">
+        <is>
           <t>via principal pavimentada</t>
         </is>
       </c>
-      <c r="Y49" t="inlineStr">
+      <c r="AD49" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z49" t="inlineStr">
+      <c r="AE49" t="inlineStr">
         <is>
           <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 13 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB49" t="inlineStr">
+      <c r="AG49" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC49" t="n">
+      <c r="AH49" t="n">
         <v>4.996865</v>
       </c>
-      <c r="AD49" t="n">
+      <c r="AI49" t="n">
         <v>-75.980124</v>
       </c>
     </row>
@@ -6513,45 +6558,45 @@
       <c r="S50" t="n">
         <v>42.5</v>
       </c>
-      <c r="V50" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W50" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X50" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>rojo, verde</t>
+        </is>
+      </c>
+      <c r="AC50" t="inlineStr">
+        <is>
           <t>via principal pavimentada</t>
         </is>
       </c>
-      <c r="Y50" t="inlineStr">
+      <c r="AD50" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z50" t="inlineStr">
+      <c r="AE50" t="inlineStr">
         <is>
           <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 28 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA50" t="inlineStr">
+      <c r="AF50" t="inlineStr">
         <is>
           <t>La Celia-Balboa</t>
         </is>
       </c>
-      <c r="AB50" t="inlineStr">
+      <c r="AG50" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC50" t="n">
+      <c r="AH50" t="n">
         <v>4.993201</v>
       </c>
-      <c r="AD50" t="n">
+      <c r="AI50" t="n">
         <v>-75.981357</v>
       </c>
     </row>
@@ -6637,40 +6682,40 @@
       <c r="S51" t="n">
         <v>17.5</v>
       </c>
-      <c r="V51" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W51" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X51" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC51" t="inlineStr">
+        <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y51" t="inlineStr">
+      <c r="AD51" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z51" t="inlineStr">
+      <c r="AE51" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 121 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB51" t="inlineStr">
+      <c r="AG51" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC51" t="n">
+      <c r="AH51" t="n">
         <v>5.063056</v>
       </c>
-      <c r="AD51" t="n">
+      <c r="AI51" t="n">
         <v>-75.99972200000001</v>
       </c>
     </row>
@@ -6756,45 +6801,45 @@
       <c r="S52" t="n">
         <v>44</v>
       </c>
-      <c r="V52" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W52" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X52" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB52" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC52" t="inlineStr">
+        <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y52" t="inlineStr">
+      <c r="AD52" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z52" t="inlineStr">
+      <c r="AE52" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 6 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA52" t="inlineStr">
+      <c r="AF52" t="inlineStr">
         <is>
           <t>Carrera 7</t>
         </is>
       </c>
-      <c r="AB52" t="inlineStr">
+      <c r="AG52" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC52" t="n">
+      <c r="AH52" t="n">
         <v>5.072806629</v>
       </c>
-      <c r="AD52" t="n">
+      <c r="AI52" t="n">
         <v>-75.96351957</v>
       </c>
     </row>
@@ -6880,45 +6925,45 @@
       <c r="S53" t="n">
         <v>44</v>
       </c>
-      <c r="V53" t="inlineStr">
+      <c r="X53" t="inlineStr">
         <is>
           <t>Afectación parcial</t>
         </is>
       </c>
-      <c r="W53" t="inlineStr">
+      <c r="Y53" t="inlineStr">
         <is>
           <t>Moderado</t>
         </is>
       </c>
-      <c r="X53" t="inlineStr">
+      <c r="AC53" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y53" t="inlineStr">
+      <c r="AD53" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z53" t="inlineStr">
+      <c r="AE53" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 18 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA53" t="inlineStr">
+      <c r="AF53" t="inlineStr">
         <is>
           <t>Calle 5</t>
         </is>
       </c>
-      <c r="AB53" t="inlineStr">
+      <c r="AG53" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC53" t="n">
+      <c r="AH53" t="n">
         <v>5.00296197</v>
       </c>
-      <c r="AD53" t="n">
+      <c r="AI53" t="n">
         <v>-76.00271345</v>
       </c>
     </row>
@@ -7004,40 +7049,40 @@
       <c r="S54" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="V54" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W54" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X54" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>rojo</t>
+        </is>
+      </c>
+      <c r="AC54" t="inlineStr">
+        <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y54" t="inlineStr">
+      <c r="AD54" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z54" t="inlineStr">
+      <c r="AE54" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 1 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB54" t="inlineStr">
+      <c r="AG54" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC54" t="n">
+      <c r="AH54" t="n">
         <v>4.885083</v>
       </c>
-      <c r="AD54" t="n">
+      <c r="AI54" t="n">
         <v>-75.97331699999999</v>
       </c>
     </row>
@@ -7123,40 +7168,40 @@
       <c r="S55" t="n">
         <v>55.7</v>
       </c>
-      <c r="V55" t="inlineStr">
+      <c r="X55" t="inlineStr">
         <is>
           <t>Riesgo inminente de colapso</t>
         </is>
       </c>
-      <c r="W55" t="inlineStr">
+      <c r="Y55" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X55" t="inlineStr">
+      <c r="AC55" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y55" t="inlineStr">
+      <c r="AD55" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z55" t="inlineStr">
+      <c r="AE55" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 9 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB55" t="inlineStr">
+      <c r="AG55" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC55" t="n">
+      <c r="AH55" t="n">
         <v>4.806935893</v>
       </c>
-      <c r="AD55" t="n">
+      <c r="AI55" t="n">
         <v>-75.74500842</v>
       </c>
     </row>
@@ -7242,40 +7287,40 @@
       <c r="S56" t="n">
         <v>55.7</v>
       </c>
-      <c r="V56" t="inlineStr">
+      <c r="X56" t="inlineStr">
         <is>
           <t>Riesgo inminente de colapso</t>
         </is>
       </c>
-      <c r="W56" t="inlineStr">
+      <c r="Y56" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X56" t="inlineStr">
+      <c r="AC56" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
         </is>
       </c>
-      <c r="Y56" t="inlineStr">
+      <c r="AD56" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z56" t="inlineStr">
+      <c r="AE56" t="inlineStr">
         <is>
           <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 147 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB56" t="inlineStr">
+      <c r="AG56" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC56" t="n">
+      <c r="AH56" t="n">
         <v>4.819139218</v>
       </c>
-      <c r="AD56" t="n">
+      <c r="AI56" t="n">
         <v>-75.76076208000001</v>
       </c>
     </row>
@@ -7361,45 +7406,45 @@
       <c r="S57" t="n">
         <v>43.1</v>
       </c>
-      <c r="V57" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W57" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X57" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB57" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC57" t="inlineStr">
+        <is>
           <t>via terciaria</t>
         </is>
       </c>
-      <c r="Y57" t="inlineStr">
+      <c r="AD57" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z57" t="inlineStr">
+      <c r="AE57" t="inlineStr">
         <is>
           <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 20 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA57" t="inlineStr">
+      <c r="AF57" t="inlineStr">
         <is>
           <t>Al Español</t>
         </is>
       </c>
-      <c r="AB57" t="inlineStr">
+      <c r="AG57" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC57" t="n">
+      <c r="AH57" t="n">
         <v>4.932181</v>
       </c>
-      <c r="AD57" t="n">
+      <c r="AI57" t="n">
         <v>-75.698198</v>
       </c>
     </row>
@@ -7485,40 +7530,40 @@
       <c r="S58" t="n">
         <v>43.1</v>
       </c>
-      <c r="V58" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W58" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X58" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB58" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC58" t="inlineStr">
+        <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y58" t="inlineStr">
+      <c r="AD58" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z58" t="inlineStr">
+      <c r="AE58" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 30 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB58" t="inlineStr">
+      <c r="AG58" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC58" t="n">
+      <c r="AH58" t="n">
         <v>4.884255</v>
       </c>
-      <c r="AD58" t="n">
+      <c r="AI58" t="n">
         <v>-75.634398</v>
       </c>
     </row>
@@ -7604,45 +7649,45 @@
       <c r="S59" t="n">
         <v>0.8</v>
       </c>
-      <c r="V59" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W59" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X59" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB59" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC59" t="inlineStr">
+        <is>
           <t>via principal pavimentada</t>
         </is>
       </c>
-      <c r="Y59" t="inlineStr">
+      <c r="AD59" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z59" t="inlineStr">
+      <c r="AE59" t="inlineStr">
         <is>
           <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 14 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA59" t="inlineStr">
+      <c r="AF59" t="inlineStr">
         <is>
           <t>Carrera 15</t>
         </is>
       </c>
-      <c r="AB59" t="inlineStr">
+      <c r="AG59" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC59" t="n">
+      <c r="AH59" t="n">
         <v>4.865108</v>
       </c>
-      <c r="AD59" t="n">
+      <c r="AI59" t="n">
         <v>-75.62179101</v>
       </c>
     </row>
@@ -7728,45 +7773,45 @@
       <c r="S60" t="n">
         <v>44.4</v>
       </c>
-      <c r="V60" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W60" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X60" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB60" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC60" t="inlineStr">
+        <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y60" t="inlineStr">
+      <c r="AD60" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z60" t="inlineStr">
+      <c r="AE60" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 135 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA60" t="inlineStr">
+      <c r="AF60" t="inlineStr">
         <is>
           <t>A Campoalegre</t>
         </is>
       </c>
-      <c r="AB60" t="inlineStr">
+      <c r="AG60" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC60" t="n">
+      <c r="AH60" t="n">
         <v>4.914981371</v>
       </c>
-      <c r="AD60" t="n">
+      <c r="AI60" t="n">
         <v>-75.61788369</v>
       </c>
     </row>
@@ -7852,40 +7897,40 @@
       <c r="S61" t="n">
         <v>44.4</v>
       </c>
-      <c r="V61" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W61" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X61" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB61" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC61" t="inlineStr">
+        <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y61" t="inlineStr">
+      <c r="AD61" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z61" t="inlineStr">
+      <c r="AE61" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 55 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB61" t="inlineStr">
+      <c r="AG61" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC61" t="n">
+      <c r="AH61" t="n">
         <v>4.966084</v>
       </c>
-      <c r="AD61" t="n">
+      <c r="AI61" t="n">
         <v>-75.63563000000001</v>
       </c>
     </row>
@@ -7971,40 +8016,40 @@
       <c r="S62" t="n">
         <v>22.4</v>
       </c>
-      <c r="V62" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
-      <c r="W62" t="inlineStr">
-        <is>
-          <t>Sin afectación</t>
-        </is>
-      </c>
       <c r="X62" t="inlineStr">
         <is>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB62" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
+        </is>
+      </c>
+      <c r="AC62" t="inlineStr">
+        <is>
           <t>camino rural sin categoria</t>
         </is>
       </c>
-      <c r="Y62" t="inlineStr">
+      <c r="AD62" t="inlineStr">
         <is>
           <t>difícil</t>
         </is>
       </c>
-      <c r="Z62" t="inlineStr">
+      <c r="AE62" t="inlineStr">
         <is>
           <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 81 m de esa vía.</t>
         </is>
       </c>
-      <c r="AB62" t="inlineStr">
+      <c r="AG62" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC62" t="n">
+      <c r="AH62" t="n">
         <v>4.783364</v>
       </c>
-      <c r="AD62" t="n">
+      <c r="AI62" t="n">
         <v>-75.641834</v>
       </c>
     </row>
@@ -8090,50 +8135,50 @@
       <c r="S63" t="n">
         <v>22.4</v>
       </c>
-      <c r="V63" t="inlineStr">
+      <c r="X63" t="inlineStr">
         <is>
           <t>Riesgo inminente de colapso</t>
         </is>
       </c>
-      <c r="W63" t="inlineStr">
+      <c r="Y63" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="X63" t="inlineStr">
+      <c r="AC63" t="inlineStr">
         <is>
           <t>via terciaria</t>
         </is>
       </c>
-      <c r="Y63" t="inlineStr">
+      <c r="AD63" t="inlineStr">
         <is>
           <t>fácil</t>
         </is>
       </c>
-      <c r="Z63" t="inlineStr">
+      <c r="AE63" t="inlineStr">
         <is>
           <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 3 m de esa vía.</t>
         </is>
       </c>
-      <c r="AA63" t="inlineStr">
+      <c r="AF63" t="inlineStr">
         <is>
           <t>Carrera 20</t>
         </is>
       </c>
-      <c r="AB63" t="inlineStr">
+      <c r="AG63" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="AC63" t="n">
+      <c r="AH63" t="n">
         <v>4.803937</v>
       </c>
-      <c r="AD63" t="n">
+      <c r="AI63" t="n">
         <v>-75.699062</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD63"/>
+  <autoFilter ref="A1:AI63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8144,7 +8189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8171,7 +8216,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
     </row>
@@ -8235,115 +8280,127 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Cuadrilla</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Días</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Sedes</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Horas de carretera</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Km</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Noches fuera</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Noches de hotel</t>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Cada columna dice de dónde viene el dato. «No reportó al MEN» no quiere decir que la sede no tenga daño: quiere decir que no hay reporte. Todas las sedes del plan se visitan, tengan o no reporte o concepto técnico.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>13</v>
-      </c>
-      <c r="C10" t="n">
-        <v>20</v>
-      </c>
-      <c r="D10" t="n">
-        <v>23.1</v>
-      </c>
-      <c r="E10" t="n">
-        <v>649</v>
-      </c>
-      <c r="F10" t="n">
-        <v>12</v>
-      </c>
-      <c r="G10" t="n">
-        <v>14</v>
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Cuadrilla</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Días</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Sedes</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Horas de carretera</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Km</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Noches fuera</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Noches de hotel</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>13</v>
+      </c>
+      <c r="C11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>649</v>
+      </c>
+      <c r="F11" t="n">
         <v>12</v>
       </c>
-      <c r="C11" t="n">
-        <v>22</v>
-      </c>
-      <c r="D11" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="E11" t="n">
-        <v>129</v>
-      </c>
-      <c r="F11" t="n">
-        <v>9</v>
-      </c>
       <c r="G11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>12</v>
       </c>
       <c r="C12" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D12" t="n">
-        <v>16.2</v>
+        <v>6.1</v>
       </c>
       <c r="E12" t="n">
-        <v>447</v>
+        <v>129</v>
       </c>
       <c r="F12" t="n">
         <v>9</v>
       </c>
       <c r="G12" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="n">
+        <v>20</v>
+      </c>
+      <c r="D13" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>447</v>
+      </c>
+      <c r="F13" t="n">
+        <v>9</v>
+      </c>
+      <c r="G13" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>